<commit_message>
Complete the clinical panel from Thera-SAbDab
Supplementary Table S5 now carries VH and VL sequences, format, developer, cognate
target, and the highest clinical trial and status as of February 2025, retrieved from
the Thera-SAbDab sequence release. No placeholders remain.

Thera-SAbDab independently confirms the Fv-identity finding: its entries for eclutatug
and lixudebart carry byte-identical VH (119 aa) and VL (107 aa), so the identical
AlphaFold3 metrics are the correct deterministic result and the pair is a valid
determinism control.

Also corrects the panel description: six whole monoclonal antibodies, two antibody-drug
conjugates and one bispecific scFv-scFv-scFc, not nine monoclonal antibodies.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Supplementary_Tables_S1-S8.xlsx
+++ b/results/Supplementary_Tables_S1-S8.xlsx
@@ -50470,7 +50470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:S10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50481,75 +50481,90 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>TheraSAbDab_entry</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Company_code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Developer</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Modality</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Cognate_target</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Cognate_target_source</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Highest_clinical_phase</t>
+          <t>TheraSAbDab_target_annotation</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Highest_clinical_trial_Feb2025</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status_Feb2025</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Year_proposed</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>VH_sequence</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>VL_sequence</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Cognate_score</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Top_scoring_antigen</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Top_score</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Cognate_rank_of_25</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Cognate_is_top_ranked</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>VH_sequence</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>VL_sequence</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Reference_urls</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -50563,71 +50578,84 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Eclutatug</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>ALE.C04 / ALE.F02</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Alentis Therapeutics AG</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Naked (unconjugated) humanized IgG1-kappa monoclonal antibody, produce</t>
+          <t>INSERM;The Mount Sinai Hospital;University of Strasbourg;Alentis Therapeutics</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>Whole mAb</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>CLDN1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>WHO INN list entry; pipeline source MAB_ON_TARGETS</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Phase 1/2 (NCT06054477, first-in-human, R/M HNSCC, monotherapy and with pembroli</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
+          <t>CLDN1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Phase-I/II</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>EVQLVESGGGLVKPGGSLRLSCAASGFSFSSYGMNWVRQAPGKGLEWVSSISPSGSYFYYADSVKGRFTISRDNAKNSLYLQMNSLRAEDTAVYYCARLPGFNPPFDHWGQGTLVTVSS</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>DIQMTQSPATLSVSPGERATLSCKASQNVGGNVDWYQWKPGQAPRLLIYGASNRYTGIPARFRGSGSGTEFTLTISSLQSEDFAVYYCLQYKNNPWTFGQGTKVEIK</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
         <v>0.512</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>CLDN6</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="O2" t="n">
         <v>0.662</v>
       </c>
-      <c r="K2" t="n">
+      <c r="P2" t="n">
         <v>4</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/pl131.pdf; https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/rl93.pdf; https://api-evsrest.nci.nih.gov/api/v1/concept/ncit/C201755?include=full</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Fv-identical Fc-variant pair (L234F/L235E/P331S); collapsed to one row</t>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab (sequences, format, clinical status as of Feb 2025); WHO INN lists and company records for target and code name</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Fv-identical Fc-variant pair: eclutatug (ALE.C04) and lixudebart (ALE.F02) share byte-identical VH (119 aa) and VL (107 aa) per Thera-SAbDab, differing only in the IgG1 Fc (L234F/L235E/P331S); collapsed to one row and used as a determinism control</t>
         </is>
       </c>
     </row>
@@ -50639,69 +50667,86 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Garetatug</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>SHR-A1904</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Jiangsu Hengrui Pharmaceuticals Co., Ltd.</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Naked humanized IgG1-kappa monoclonal antibody (the INN "garetatug" de</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>Whole mAb ADC</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>CLDN18.2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>WHO INN list entry; pipeline source MAB_ON_TARGETS</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Phase 3 (as the ADC garetatug rezetecan / SHR-A1904)</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
+          <t>CLDN18</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>EVQLVQSGAEVKKPGASVKVSCKASGYTFTSYWMHWVRQAPGQRLEWMGMIHPNSGSTNYNEKFKGRVTITRDTSASTAYMELSSLRSEDTAVYYCARLKTGNSFDYWGQGTTVTVSS</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>DIVLTQSPDSLAVSLGERATINCKSSQSLLNSGNQKNYLTWYQQKPGQPPKLLIYWASTRESGVPDRFSGSGSGTDFTLTISSLQAEDVAVYYCQNAYTYPFTFGQGTKLEIK</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
         <v>0.887</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>CLDN18.2</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="O3" t="n">
         <v>0.887</v>
       </c>
-      <c r="K3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/rl94.pdf; https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/pl132.pdf; https://clinicaltrials.gov/study/NCT06649292</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab (sequences, format, clinical status as of Feb 2025); WHO INN lists and company records for target and code name</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab annotates the target at gene level (CLDN18); the therapeutic target is the isoform CLDN18.2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -50711,69 +50756,86 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Omectatug</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>ASKB589</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Jiangsu Aosaikang Pharmaceutical Co., Ltd.</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Naked (unconjugated) humanized IgG1-kappa monoclonal antibody; afucosy</t>
+          <t>AskGene Pharma;Jiangsu Aosaikang Pharmaceutical</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>Whole mAb</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>CLDN18.2</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>WHO INN list entry; pipeline source MAB_ON_TARGETS</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Phase 3 (ongoing/active, not recruiting) — NCT06206733, first-line advanced/meta</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
+          <t>CLDN18</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Phase-III</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>QVQLVQSGAEVKKPGASVKVSCKASGYTFTSYVINWVRQATGQGLEWIGEIHPRGGNTYYSEKFRGRVTLTADTSISTAYMELSSLRSEDTAVYYCARLRRGNAMDYWDQGTTVTVSS</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>DIVMTQSPSSLAVSLGEMATINCKSSQSLLNSGNQRNYLTWYQQKPGQPPKLLIYWASTRESGVPDRFSGSGSGTDFTLTISSLQAEDVAVYYCQNSYNYPYTFGQGTKLERK</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
         <v>0.839</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>CLDN18.2</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="O4" t="n">
         <v>0.839</v>
       </c>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/pl131.pdf; https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/rl93.pdf; https://pubchem.ncbi.nlm.nih.gov/rest/pug/substance/name/omectatug/synonyms/TXT</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab (sequences, format, clinical status as of Feb 2025); WHO INN lists and company records for target and code name</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab annotates the target at gene level (CLDN18); the therapeutic target is the isoform CLDN18.2</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -50783,69 +50845,86 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Tecotabart</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>LM-302</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>LaNova Medicines</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Humanized IgG1-kappa monoclonal antibody (produced in CHO-K1, glycofor</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>Whole mAb</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>CLDN18.2</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>WHO INN list entry; pipeline source MAB_ON_TARGETS</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Phase 3 (two registered Phase III trials in CLDN18</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
+          <t>CLDN18</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Phase-I/II</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>EVQLVESGGGLVQPGGSLRLSCAASGFTFSTFGMHWVRQAPGKGLEWVSYITSGESPIYFTDTVKGRFTISRDNAKNSLYLQMNSLRAEDTAVYYCARSSYYGNSMDYWGQGTLVTVSS</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>DIVMTQSPDSLAVSLGERATINCRSSQSLLNAGNRKNYLTWYQQKPGQPPKLLIYWASTRESGVPDRFSGSGSGTDFTLTISSLQAEDVAVYYCQNAYSYPFTFGGGTKLEIK</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
         <v>0.354</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>CLDN5</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="O5" t="n">
         <v>0.727</v>
       </c>
-      <c r="K5" t="n">
+      <c r="P5" t="n">
         <v>15</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/rl92.pdf; https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/pl130.pdf; https://gsrs.ncats.nih.gov/ginas/app/beta/substances/9GK5GYD8DQ</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab (sequences, format, clinical status as of Feb 2025); WHO INN lists and company records for target and code name</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab annotates the target at gene level (CLDN18); the therapeutic target is the isoform CLDN18.2</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -50855,69 +50934,86 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Gresonitamab</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>AMG 910</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Amgen Inc.</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bispecific T-cell engager (half-life-extended BiTE); WHO INN format: s</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>Bispecific scFv-scFv-scFc</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>CLDN18.2</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>WHO INN list entry; pipeline source MAB_ON_TARGETS</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Phase 1 (terminated)</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
+          <t>CLDN18;CD3E</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Phase-I</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Discontinued</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>2021</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>QVQLVQSGAEVKKPGASVKVSCKASGYTFTGYYMHWVRQAPGQCLEWMGWINPNSGGTKYAQKFQGRVTMTRDTSISTAYMELSRLRSDDTAVYYCARDRITVAGTYYYYGMDVWGQGTTVTVSS</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>DIQMTQSPSSVSASVGDRVTITCRASQGVNNWLAWYQQKPGKAPKLLIYTASSLQSGVPSRFSGSGSGTDFTLTIRSLQPEDFATYYCQQANSFPITFGCGTRLEIK</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
         <v>0.398</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>CLDN3</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="O6" t="n">
         <v>0.779</v>
       </c>
-      <c r="K6" t="n">
+      <c r="P6" t="n">
         <v>16</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/rl87.pdf; https://clinicaltrials.gov/study/NCT04260191; https://clinicaltrials.gov/api/v2/studies/NCT04260191?fields=NCTId,BriefTitle,OverallStatus,Phase,LeadSponsorName,InterventionName,InterventionOtherName,Condition,CompletionDate,WhyStopped</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab (sequences, format, clinical status as of Feb 2025); WHO INN lists and company records for target and code name</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab annotates the target at gene level (CLDN18); the therapeutic target is the isoform CLDN18.2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -50927,69 +51023,86 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>Osemitamab</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>TST001</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Transcenta Holding Ltd.</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Naked (unconjugated) humanized IgG1-kappa monoclonal antibody, ADCC-en</t>
+          <t>Transcenta</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>Whole mAb</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>CLDN18.2</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>WHO INN list entry; pipeline source MAB_ON_TARGETS</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
+          <t>CLDN18</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Phase-II</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>2022</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>QVQLVQSGAEVKKPGASVKVSCKASGYTFTGYNMNWVRQAPGQGLEWMGNIDPYYGGTSYNQKFKGRVTMTIDKSTSTVYMELSSLRSEDTAVYYCARMYHGNAFDYWGQGTTVTVSS</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>DIVMTQSPDSLAVSLGERATINCKSSQSLLNSGNLKNYLTWYQQKPGQPPKLLIYWASTRKSGVPDRFSGSGSGTDFTLTISSLQAEDVAVYYCQNDYSYPLTFGGGTKVEIK</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
         <v>0.378</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>CLDN9</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="O7" t="n">
         <v>0.735</v>
       </c>
-      <c r="K7" t="n">
+      <c r="P7" t="n">
         <v>21</v>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/pl126.pdf; https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/rl88.pdf; https://clinicaltrials.gov/study/NCT06093425</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab (sequences, format, clinical status as of Feb 2025); WHO INN lists and company records for target and code name</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab annotates the target at gene level (CLDN18); the therapeutic target is the isoform CLDN18.2</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -50997,69 +51110,82 @@
           <t>sonesitatug vedotin</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>None - no substance with this INN exists.</t>
-        </is>
-      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sonesitatug</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>N/A - "sonesitamab" does not exist as an INN. (Nearest real INN, sones</t>
+          <t>KeyMed Biosciences;Miracogen;AstraZeneca</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>Whole mAb</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>CLDN18.2</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>WHO INN / AdisInsight (INN corrected from the misspelling "sonesitamab")</t>
-        </is>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>N/A - no drug named "sonesitamab" is registered in ClinicalTrials</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
+          <t>CLDN18</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Phase-III</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>QVQLQESGPGLVKPSETLSLTCTVSGGSISSNYAWNWIRQPPGKGLEWIGYIYYSGNTNYNPSLKSRVTISRDTSKNQFSLKLSSVTAADTAVYYCATSYYGNSFIYWGQGTLVTVSS</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>DIVMTQSPDSLAVSLGERATINCKSSQSLLNSGNQKNYLTWYQQKPGQPPKLLIYWASTRESGVPDRFSGSGSGTDFTLTISSLQAEDVAVYYCQNAYSFPWTFGQGTKVEIK</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
         <v>0.363</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>CLDN11</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="O8" t="n">
         <v>0.544</v>
       </c>
-      <c r="K8" t="n">
+      <c r="P8" t="n">
         <v>21</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/pl131.pdf; https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/rl93.pdf; https://opig.stats.ox.ac.uk/webapps/sabdab-sabpred/therasabdab/search/?therapeutic=sonesitamab</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Source tables use the misspelling "sonesitamab"; correct INN is sonesitatug vedotin (CMG901/AZD0901, KYM Biosciences/AstraZeneca), anti-CLDN18.2 ADC, Phase 3</t>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab (sequences, format, clinical status as of Feb 2025); WHO INN lists and company records for target and code name</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Source tables use the misspelling 'sonesitamab'; correct INN is sonesitatug (sonesitatug vedotin, CMG901/AZD0901)</t>
         </is>
       </c>
     </row>
@@ -51071,69 +51197,86 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Zolbetuximab</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>IMAB362</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Astellas Pharma</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Naked (unconjugated) chimeric mouse/human IgG1 monoclonal antibody; cy</t>
+          <t>Ganymed Pharmaceuticals</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>Whole mAb</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>CLDN18.2</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>WHO INN list entry; pipeline source MAB_ON_TARGETS</t>
-        </is>
-      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phase 3 completed and approved/marketed — brand name VYLOY (zolbetuximab-clzb); </t>
-        </is>
-      </c>
-      <c r="H9" t="n">
+          <t>CLDN18</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>2017</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>QVQLQQPGAELVRPGASVKLSCKASGYTFTSYWINWVKQRPGQGLEWIGNIYPSDSYTNYNQKFKDKATLTVDKSSSTAYMQLSSPTSEDSAVYYCTRSWRGNSFDYWGQGTTLTVSS</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>DIVMTQSPSSLTVTAGEKVTMSCKSSQSLLNSGNQKNYLTWYQQKPGQPPKLLIYWASTRESGVPDRFTGSGSGTDFTLTISSVQAEDLAVYYCQNDYSYPFTFGSGTKLEIK</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
         <v>0.273</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>CLDN5</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="O9" t="n">
         <v>0.805</v>
       </c>
-      <c r="K9" t="n">
+      <c r="P9" t="n">
         <v>24</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>https://www.fda.gov/drugs/resources-information-approved-drugs/fda-approves-zolbetuximab-clzb-chemotherapy-gastric-or-gastroesophageal-junction-adenocarcinoma; https://www.accessdata.fda.gov/drugsatfda_docs/label/2024/761365s000lbl.pdf; https://newsroom.astellas.com/2024-09-24-Astellas-Receives-Approval-from-the-European-Commission-for-VYLOYTM-zolbetuximab-in-Combination-with-Chemotherapy-for-Advanced-Gastric-and-Gastroesophageal-Junction-Cancer</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab (sequences, format, clinical status as of Feb 2025); WHO INN lists and company records for target and code name</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab annotates the target at gene level (CLDN18); the therapeutic target is the isoform CLDN18.2</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -51143,69 +51286,82 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>Ixotatug</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>TORL-1-23</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>TORL BioTherapeutics, LLC</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Humanized/chimeric IgG1-kappa monoclonal antibody. The unconjugated an</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>Whole mAb ADC</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>CLDN6</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>WHO INN list entry; pipeline source MAB_ON_TARGETS</t>
-        </is>
-      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Phase 2 (registrational/pivotal)</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
+          <t>CLDN6</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>2025</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>EVQLLESGGGLVQPGGSMRLSCAASGFTFSNYWMNWVRQAPGKGLEWVAQIRLKSDNYATHYADSVKGRFTISRDDSKNTVYLQMNSLRAEDTGVYYCNDGPPSGSWGQGTLLTVSS</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>DIQMTQSPSSLSASVGDRVTITCRISENIYSYLAWYQQKPGKAPKLLVYNAKILVEGVPSRFSGSGSGTDFTLTISSLQPEDFGTYYCQHHYTVPWTFGQGTKLEIK</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
         <v>0.445</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>CLDN25</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="O10" t="n">
         <v>0.738</v>
       </c>
-      <c r="K10" t="n">
+      <c r="P10" t="n">
         <v>9</v>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>&lt;&lt;AUTHOR: paste from Thera-SAbDab&gt;&gt;</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/pl132.pdf; https://cdn.who.int/media/docs/default-source/international-nonproprietary-names-(inn)/rl94.pdf; https://clinicaltrials.gov/study/NCT06690775</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Thera-SAbDab (sequences, format, clinical status as of Feb 2025); WHO INN lists and company records for target and code name</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>